<commit_message>
Add README.md and update AE2 and AE3 Excel files for project documentation
</commit_message>
<xml_diff>
--- a/static/informes/Ae2.xlsx
+++ b/static/informes/Ae2.xlsx
@@ -484,7 +484,7 @@
       </c>
       <c r="C9" s="1" t="inlineStr">
         <is>
-          <t>FECHA:10-5-2026</t>
+          <t>FECHA:11-5-2026</t>
         </is>
       </c>
     </row>
@@ -905,7 +905,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t xml:space="preserve">                           profesor                                                               administrador</t>
+          <t xml:space="preserve">                           profesor                                                               admin</t>
         </is>
       </c>
     </row>

</xml_diff>